<commit_message>
002 3.0: tensores de muros anclados en el larguero de 0.60 m
Los tensores 845-852 de los muros A y B regresan al larguero de 0.60 m
(como en el modelo del usuario) en lugar de la base de las columnas.
Mismos perfiles. CUT OFF 43, factores X 1.0973 / Z 1.0183.
6673.62 kg, 43.45 kg/m2 con 5% de conexiones. Se regeneran hoja de
sismo y viento, áreas tributarias, DXF, desglose y reacciones.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DbpSpoM7qi5cJ9LMKpwgVv
</commit_message>
<xml_diff>
--- a/002/002_AreasTributarias_NOSE_DOCK_H5_H6_3.0.xlsx
+++ b/002/002_AreasTributarias_NOSE_DOCK_H5_H6_3.0.xlsx
@@ -1930,7 +1930,7 @@
     <t xml:space="preserve">SELFWEIGHT Z 1</t>
   </si>
   <si>
-    <t xml:space="preserve">CASO 4: estas líneas van ANTES del SPECTRUM. CASOS 5 A 7 usan la masa del caso 4. Cubierta y muros quedan como JOINT LOAD en las cabezas de columna. CUT OFF MODE SHAPE = 43; participación modal acumulada X = 92.03% y Z = 95.93%. Los muros van a cada cabeza con la mitad de cada claro (8 m) y se escalan al total de muros de la hoja de sismo (2,698.6 kg con la cortina).</t>
+    <t xml:space="preserve">CASO 4: estas líneas van ANTES del SPECTRUM. CASOS 5 A 7 usan la masa del caso 4. Cubierta y muros quedan como JOINT LOAD en las cabezas de columna. CUT OFF MODE SHAPE = 43; participación modal acumulada X = 91.73% y Z = 96.12%. Los muros van a cada cabeza con la mitad de cada claro (8 m) y se escalan al total de muros de la hoja de sismo (2,698.6 kg con la cortina).</t>
   </si>
   <si>
     <t xml:space="preserve">RESUMEN — ÁREAS, CARGAS TOTALES Y PESO SÍSMICO W</t>
@@ -2224,7 +2224,7 @@
     <t xml:space="preserve">T_B en X (modo con más masa en X)</t>
   </si>
   <si>
-    <t xml:space="preserve">Modo 1: mayor participación en X (82.16%).</t>
+    <t xml:space="preserve">Modo 1: mayor participación en X (81.83%).</t>
   </si>
   <si>
     <t xml:space="preserve">motor 3.0 (43 modos)</t>
@@ -2233,7 +2233,7 @@
     <t xml:space="preserve">T_B en Z (modo con más masa en Z)</t>
   </si>
   <si>
-    <t xml:space="preserve">Modo 7: mayor participación en Z (88.92%).</t>
+    <t xml:space="preserve">Modo 7: mayor participación en Z (88.23%).</t>
   </si>
   <si>
     <t xml:space="preserve">V_est en X = máx(Cs(T_B), 0.8·Cs(T_A))·W</t>
@@ -2269,13 +2269,13 @@
     <t xml:space="preserve">Factor del SPECTRUM en X</t>
   </si>
   <si>
-    <t xml:space="preserve">Factor mínimo requerido en X; el .STD usa 1.0929.</t>
+    <t xml:space="preserve">Factor mínimo requerido en X; el .STD usa 1.0973.</t>
   </si>
   <si>
     <t xml:space="preserve">Factor del SPECTRUM en Z</t>
   </si>
   <si>
-    <t xml:space="preserve">Factor mínimo requerido en Z; el .STD usa 1.0108.</t>
+    <t xml:space="preserve">Factor mínimo requerido en Z; el .STD usa 1.0183.</t>
   </si>
 </sst>
 </file>
@@ -18338,13 +18338,13 @@
         <v>688</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>149.8744</v>
+        <v>146.2814</v>
       </c>
       <c r="D34" s="33" t="n">
         <v>1.2668</v>
       </c>
       <c r="E34" s="19" t="n">
-        <v>148.722</v>
+        <v>145.157</v>
       </c>
       <c r="F34" s="10" t="s">
         <v>689</v>
@@ -18373,12 +18373,12 @@
       </c>
       <c r="C36" s="11" t="n">
         <f aca="false">SUM(C23:C35)</f>
-        <v>917.9997</v>
+        <v>914.4067</v>
       </c>
       <c r="D36" s="8"/>
       <c r="E36" s="19" t="n">
         <f aca="false">SUM(E23:E35)</f>
-        <v>6677.186</v>
+        <v>6673.621</v>
       </c>
       <c r="F36" s="10" t="s">
         <v>693</v>
@@ -18474,7 +18474,7 @@
       </c>
       <c r="C40" s="11" t="n">
         <f aca="false">E36/1000</f>
-        <v>6.677186</v>
+        <v>6.673621</v>
       </c>
       <c r="D40" s="8" t="s">
         <v>696</v>
@@ -18674,7 +18674,7 @@
       </c>
       <c r="C45" s="11" t="n">
         <f aca="false">SUM(C40:C44)</f>
-        <v>12.403963112</v>
+        <v>12.400398112</v>
       </c>
       <c r="D45" s="8" t="s">
         <v>696</v>
@@ -18746,7 +18746,7 @@
         <v>710</v>
       </c>
       <c r="C46" s="11" t="n">
-        <v>12.37314</v>
+        <v>12.41839</v>
       </c>
       <c r="D46" s="8" t="s">
         <v>696</v>
@@ -18948,7 +18948,7 @@
         <v>731</v>
       </c>
       <c r="C59" s="11" t="n">
-        <v>0.6197</v>
+        <v>0.61943</v>
       </c>
       <c r="D59" s="8" t="s">
         <v>720</v>
@@ -18965,7 +18965,7 @@
         <v>734</v>
       </c>
       <c r="C60" s="11" t="n">
-        <v>0.37184</v>
+        <v>0.38249</v>
       </c>
       <c r="D60" s="8" t="s">
         <v>720</v>
@@ -18982,7 +18982,7 @@
         <v>736</v>
       </c>
       <c r="C61" s="11" t="n">
-        <v>2075.24562</v>
+        <v>2082.83504</v>
       </c>
       <c r="D61" s="8" t="s">
         <v>58</v>
@@ -18999,7 +18999,7 @@
         <v>738</v>
       </c>
       <c r="C62" s="11" t="n">
-        <v>2121.10971</v>
+        <v>2128.86686</v>
       </c>
       <c r="D62" s="8" t="s">
         <v>58</v>
@@ -19016,7 +19016,7 @@
         <v>739</v>
       </c>
       <c r="C63" s="11" t="n">
-        <v>1867.72106</v>
+        <v>1874.55153</v>
       </c>
       <c r="D63" s="8" t="s">
         <v>58</v>
@@ -19033,7 +19033,7 @@
         <v>741</v>
       </c>
       <c r="C64" s="11" t="n">
-        <v>1908.99874</v>
+        <v>1915.98017</v>
       </c>
       <c r="D64" s="8" t="s">
         <v>58</v>
@@ -19050,7 +19050,7 @@
         <v>742</v>
       </c>
       <c r="C65" s="11" t="n">
-        <v>1708.95319</v>
+        <v>1708.31557</v>
       </c>
       <c r="D65" s="8" t="s">
         <v>58</v>
@@ -19067,7 +19067,7 @@
         <v>744</v>
       </c>
       <c r="C66" s="11" t="n">
-        <v>1888.63624</v>
+        <v>1881.58154</v>
       </c>
       <c r="D66" s="8" t="s">
         <v>58</v>
@@ -19085,7 +19085,7 @@
       </c>
       <c r="C67" s="11" t="n">
         <f aca="false">MAX(1,C63/C65)</f>
-        <v>1.09290358034909</v>
+        <v>1.09730986646688</v>
       </c>
       <c r="D67" s="8" t="s">
         <v>41</v>
@@ -19103,7 +19103,7 @@
       </c>
       <c r="C68" s="11" t="n">
         <f aca="false">MAX(1,C64/C66)</f>
-        <v>1.01078158915345</v>
+        <v>1.01828176418015</v>
       </c>
       <c r="D68" s="8" t="s">
         <v>41</v>

</xml_diff>

<commit_message>
002 3.0: grupos de columnas y largueros, notas de masas y referencias
Correcciones de la revisión cruzada (sin cambio de resultados):
- STD: _COLUMNAS_EJES_1_Y_3 y _COLUMNAS_EJE_2 con los miembros de cada
  eje; _LARGUEROS_AB_10M/6M pasan a _LARGUEROS_AB_C12/C23 (claros de 8 m).
- DXF: la planta de nodos da la masa total del caso 4 de cada cabeza
  (techo + muros y cortina) y la nota ya no dice que sólo va el techo.
- Áreas: notas de la hoja STAAD con la celda de MUROS que usa cada
  fórmula, encabezado de NODOS_TECHO O5 y referencia de RESUMEN B2.
- Desglose: la figura de cada familia no se separa de su pie.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DbpSpoM7qi5cJ9LMKpwgVv
</commit_message>
<xml_diff>
--- a/002/002_AreasTributarias_NOSE_DOCK_H5_H6_3.0.xlsx
+++ b/002/002_AreasTributarias_NOSE_DOCK_H5_H6_3.0.xlsx
@@ -1528,7 +1528,7 @@
     <t xml:space="preserve">CV techo (kg)</t>
   </si>
   <si>
-    <t xml:space="preserve">Línea STAAD caso 4 (masa)</t>
+    <t xml:space="preserve">Parte de techo de la línea del caso 4 (los muros y la cortina se suman en la hoja STAAD)</t>
   </si>
   <si>
     <t xml:space="preserve">Nota</t>
@@ -1789,7 +1789,7 @@
     <t xml:space="preserve">L1 con h = 1.20 m</t>
   </si>
   <si>
-    <t xml:space="preserve">CM de muros × h (MUROS P78) · Largueros y línea de 6.60 m fuera del vano (h = 1.20 m) del muro 1</t>
+    <t xml:space="preserve">CM de muros × h (MUROS P80) · Largueros y línea de 6.60 m fuera del vano (h = 1.20 m) del muro 1</t>
   </si>
   <si>
     <t xml:space="preserve">Nivel 1 (0.60 m) y L1-3.2</t>
@@ -1819,34 +1819,34 @@
     <t xml:space="preserve">L1-P (dintel puerta)</t>
   </si>
   <si>
-    <t xml:space="preserve">CM de muros × h (MUROS P81) · Dintel de la puerta a 2.40 m: de 2.40 a 2.70 m</t>
+    <t xml:space="preserve">CM de muros × h (MUROS P83) · Dintel de la puerta a 2.40 m: de 2.40 a 2.70 m</t>
   </si>
   <si>
     <t xml:space="preserve">L1-5.1, L1-5.2</t>
   </si>
   <si>
-    <t xml:space="preserve">CM de muros × h (MUROS P88) · Largueros a 5.40 m junto a la cortina</t>
+    <t xml:space="preserve">CM de muros × h (MUROS P90) · Largueros a 5.40 m junto a la cortina</t>
   </si>
   <si>
     <t xml:space="preserve">L1-6.2 (dintel)</t>
   </si>
   <si>
-    <t xml:space="preserve">CM de muros × h (MUROS P91) · Dintel de la cortina a 6.60 m (sobre el vano)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CM de muros × h (MUROS P93) · Larguero a 7.80 m del muro 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CM de muros × h (MUROS P94) · Larguero a 9.00 m del muro 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CM de muros × h (MUROS P95) · Último larguero (9.45 m) del muro 1</t>
+    <t xml:space="preserve">CM de muros × h (MUROS P93) · Dintel de la cortina a 6.60 m (sobre el vano)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CM de muros × h (MUROS P95) · Larguero a 7.80 m del muro 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CM de muros × h (MUROS P96) · Larguero a 9.00 m del muro 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CM de muros × h (MUROS P97) · Último larguero (9.45 m) del muro 1</t>
   </si>
   <si>
     <t xml:space="preserve">VM-1 (franja del muro eje 1)</t>
   </si>
   <si>
-    <t xml:space="preserve">CM de muros × h (MUROS P96) · Franja alta del muro 1 (arriba de 9.45 m) a la viga del eje 1</t>
+    <t xml:space="preserve">CM de muros × h (MUROS P98) · Franja alta del muro 1 (arriba de 9.45 m) a la viga del eje 1</t>
   </si>
   <si>
     <t xml:space="preserve">VA-1 y VB-1 (franja)</t>
@@ -1930,13 +1930,13 @@
     <t xml:space="preserve">SELFWEIGHT Z 1</t>
   </si>
   <si>
-    <t xml:space="preserve">CASO 4: estas líneas van ANTES del SPECTRUM. CASOS 5 A 7 usan la masa del caso 4. Cubierta y muros quedan como JOINT LOAD en las cabezas de columna. CUT OFF MODE SHAPE = 43; participación modal acumulada X = 91.73% y Z = 96.12%. Los muros van a cada cabeza con la mitad de cada claro (8 m) y se escalan al total de muros de la hoja de sismo (2,698.6 kg con la cortina).</t>
+    <t xml:space="preserve">CASO 4: estas líneas van ANTES del SPECTRUM. CASOS 5 A 7 usan la masa del caso 4. Cubierta y muros quedan como JOINT LOAD en las cabezas de columna. CUT OFF MODE SHAPE = 43; participación modal acumulada X = 91.73% y Z = 96.12%. Los muros van a cada cabeza con la mitad de cada claro (8 m) y se escalan al total de muros y cortina que traía el caso 4 de la R1.3_3 (2,698.6 kg).</t>
   </si>
   <si>
     <t xml:space="preserve">RESUMEN — ÁREAS, CARGAS TOTALES Y PESO SÍSMICO W</t>
   </si>
   <si>
-    <t xml:space="preserve">Totales para revisar contra STAAD (suma de cargas del caso 1) y el W que va a la hoja de espectros (DATOS C60 y C61).</t>
+    <t xml:space="preserve">Totales para revisar contra STAAD (suma de cargas del caso 1) y el W que va a la hoja de espectros (RESUMEN C45 y C46).</t>
   </si>
   <si>
     <t xml:space="preserve">1. ÁREAS TRIBUTARIAS</t>

</xml_diff>

<commit_message>
002 3.0: masa sísmica de muros con 5.85 kg/m² y muro 1 partido a la mitad
Caso 4: cada cabeza lleva el techo (19.32 kg/m² × área tributaria), los
muros A y B de 0.30 m al alero con la mitad de cada claro, y el muro 1
partido en X = 5.04 m (cada mitad con sus vanos) a los nodos 7 y 8, más
media cortina en cada jamba: 7 = 1006.45, 8 = 1033.96, 75 y 76 =
1233.64, 9 y 10 = 609.54 kg. Muros y cortina 2610.84 kg = 5.85 × 378.30
+ 397.8. Mismos perfiles; factores X 1.0983 / Z 1.0209; 43.45 kg/m2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DbpSpoM7qi5cJ9LMKpwgVv
</commit_message>
<xml_diff>
--- a/002/002_AreasTributarias_NOSE_DOCK_H5_H6_3.0.xlsx
+++ b/002/002_AreasTributarias_NOSE_DOCK_H5_H6_3.0.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1298" uniqueCount="750">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1298" uniqueCount="751">
   <si>
     <t xml:space="preserve">ÁREAS TRIBUTARIAS Y CARGAS PARA STAAD — HANGAR NOSE-DOCK H5-H6 — DATOS</t>
   </si>
@@ -1891,34 +1891,37 @@
     <t xml:space="preserve">N7</t>
   </si>
   <si>
-    <t xml:space="preserve">7 FX 1034.78 FZ 1034.78</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cubierta 389.49 kg (20.16 m², NODOS_TECHO) + muros y cortina 645.29 kg en la cabeza.</t>
+    <t xml:space="preserve">7 FX 1006.45 FZ 1006.45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cubierta 389.49 kg (20.16 m², NODOS_TECHO) + muro A 234.61 kg (Z 0 a 4 m) + mitad del muro 1 con la puerta 183.44 kg (X 0 a 5.04 m) + ½ cortina 198.90 kg.</t>
   </si>
   <si>
     <t xml:space="preserve">N8</t>
   </si>
   <si>
-    <t xml:space="preserve">8 FX 1034.78 FZ 1034.78</t>
+    <t xml:space="preserve">8 FX 1033.96 FZ 1033.96</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cubierta 389.49 kg (20.16 m², NODOS_TECHO) + muro B 234.61 kg (Z 0 a 4 m) + mitad del muro 1 210.96 kg (X 5.04 a 10.08 m) + ½ cortina 198.90 kg.</t>
   </si>
   <si>
     <t xml:space="preserve">N75, N76</t>
   </si>
   <si>
-    <t xml:space="preserve">75 76 FX 1253.24 FZ 1253.24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cubierta 778.98 kg (40.32 m², NODOS_TECHO) + muros 474.26 kg en la cabeza.</t>
+    <t xml:space="preserve">75 76 FX 1233.64 FZ 1233.64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cubierta 778.98 kg (40.32 m², NODOS_TECHO) + muro A o B 454.66 kg (Z 4 a 12 m).</t>
   </si>
   <si>
     <t xml:space="preserve">N9, N10</t>
   </si>
   <si>
-    <t xml:space="preserve">9 10 FX 619.25 FZ 619.25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cubierta 389.49 kg (20.16 m², NODOS_TECHO) + muros 229.76 kg en la cabeza.</t>
+    <t xml:space="preserve">9 10 FX 609.54 FZ 609.54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cubierta 389.49 kg (20.16 m², NODOS_TECHO) + muro A o B 220.05 kg (Z 12 a 16 m).</t>
   </si>
   <si>
     <t xml:space="preserve">SELFWEIGHT X 1</t>
@@ -1930,7 +1933,7 @@
     <t xml:space="preserve">SELFWEIGHT Z 1</t>
   </si>
   <si>
-    <t xml:space="preserve">CASO 4: estas líneas van ANTES del SPECTRUM. CASOS 5 A 7 usan la masa del caso 4. Cubierta y muros quedan como JOINT LOAD en las cabezas de columna. CUT OFF MODE SHAPE = 43; participación modal acumulada X = 91.73% y Z = 96.12%. Los muros van a cada cabeza con la mitad de cada claro (8 m) y se escalan al total de muros y cortina que traía el caso 4 de la R1.3_3 (2,698.6 kg).</t>
+    <t xml:space="preserve">CASO 4: estas líneas van ANTES del SPECTRUM. CASOS 5 A 7 usan la masa del caso 4. Cubierta y muros quedan como JOINT LOAD en las cabezas de columna. CUT OFF MODE SHAPE = 43; participación modal acumulada X = 91.66% y Z = 96.10%. Muros A y B de 0.30 m al alero con la mitad de cada claro (Z 0 a 4, 4 a 12 y 12 a 16 m); muro 1 partido a la mitad en X = 5.04 m, cada mitad con sus vanos, una al nodo 7 y otra al nodo 8; media cortina en cada jamba. Muros y cortina: 5.85 kg/m² × 378.30 m² + 397.8 kg = 2,610.84 kg.</t>
   </si>
   <si>
     <t xml:space="preserve">RESUMEN — ÁREAS, CARGAS TOTALES Y PESO SÍSMICO W</t>
@@ -2224,7 +2227,7 @@
     <t xml:space="preserve">T_B en X (modo con más masa en X)</t>
   </si>
   <si>
-    <t xml:space="preserve">Modo 1: mayor participación en X (81.83%).</t>
+    <t xml:space="preserve">Modo 1: mayor participación en X (81.76%).</t>
   </si>
   <si>
     <t xml:space="preserve">motor 3.0 (43 modos)</t>
@@ -2233,7 +2236,7 @@
     <t xml:space="preserve">T_B en Z (modo con más masa en Z)</t>
   </si>
   <si>
-    <t xml:space="preserve">Modo 7: mayor participación en Z (88.23%).</t>
+    <t xml:space="preserve">Modo 7: mayor participación en Z (88.00%).</t>
   </si>
   <si>
     <t xml:space="preserve">V_est en X = máx(Cs(T_B), 0.8·Cs(T_A))·W</t>
@@ -2269,13 +2272,13 @@
     <t xml:space="preserve">Factor del SPECTRUM en X</t>
   </si>
   <si>
-    <t xml:space="preserve">Factor mínimo requerido en X; el .STD usa 1.0973.</t>
+    <t xml:space="preserve">Factor mínimo requerido en X; el .STD usa 1.0983.</t>
   </si>
   <si>
     <t xml:space="preserve">Factor del SPECTRUM en Z</t>
   </si>
   <si>
-    <t xml:space="preserve">Factor mínimo requerido en Z; el .STD usa 1.0183.</t>
+    <t xml:space="preserve">Factor mínimo requerido en Z; el .STD usa 1.0209.</t>
   </si>
 </sst>
 </file>
@@ -17160,7 +17163,7 @@
         <v>624</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="F43" s="21" t="str">
         <f aca="false">IF(LEN($D43)&gt;79,"MÁS DE 79","")</f>
@@ -17224,16 +17227,16 @@
     </row>
     <row r="44" customFormat="false" ht="26.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="21" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="C44" s="8" t="s">
         <v>83</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="F44" s="21" t="str">
         <f aca="false">IF(LEN($D44)&gt;79,"MÁS DE 79","")</f>
@@ -17297,16 +17300,16 @@
     </row>
     <row r="45" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="21" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>83</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="F45" s="21" t="str">
         <f aca="false">IF(LEN($D45)&gt;79,"MÁS DE 79","")</f>
@@ -17321,10 +17324,10 @@
         <v>83</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="F46" s="21" t="str">
         <f aca="false">IF(LEN($D46)&gt;79,"MÁS DE 79","")</f>
@@ -17339,10 +17342,10 @@
         <v>83</v>
       </c>
       <c r="D47" s="6" t="s">
+        <v>634</v>
+      </c>
+      <c r="E47" s="9" t="s">
         <v>633</v>
-      </c>
-      <c r="E47" s="9" t="s">
-        <v>632</v>
       </c>
       <c r="F47" s="21" t="str">
         <f aca="false">IF(LEN($D47)&gt;79,"MÁS DE 79","")</f>
@@ -17356,9 +17359,9 @@
       <c r="E48" s="9"/>
       <c r="F48" s="21"/>
     </row>
-    <row r="49" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="270.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="21" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="C49" s="8"/>
       <c r="D49" s="6"/>
@@ -17536,7 +17539,7 @@
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="2" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -17545,7 +17548,7 @@
     </row>
     <row r="2" s="1" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="3" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -17555,7 +17558,7 @@
     <row r="3" s="1" customFormat="true" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="4" s="1" customFormat="true" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
@@ -17581,89 +17584,89 @@
     </row>
     <row r="6" s="1" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="C6" s="11" t="n">
         <f aca="false">TECHO!$J$20</f>
         <v>161.28</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
     </row>
     <row r="7" s="1" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C7" s="11" t="n">
         <f aca="false">MUROS!$O$41</f>
         <v>298.24016</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
     </row>
     <row r="8" s="1" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="C8" s="11" t="n">
         <f aca="false">MUROS!$O$71</f>
         <v>12.64016</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
     </row>
     <row r="9" s="1" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C9" s="11" t="n">
         <f aca="false">MUROS!$N$99</f>
         <v>67.4184</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="C10" s="11" t="n">
         <f aca="false">C7+C8+C9</f>
         <v>378.29872</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="F10" s="10" t="s">
         <v>41</v>
@@ -17783,7 +17786,7 @@
     </row>
     <row r="12" s="1" customFormat="true" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="4" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
@@ -17809,7 +17812,7 @@
     </row>
     <row r="14" s="1" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="C14" s="19" t="n">
         <f aca="false">DATOS!$C$8*C6</f>
@@ -17819,15 +17822,15 @@
         <v>58</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
     </row>
     <row r="15" s="1" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C15" s="19" t="n">
         <f aca="false">DATOS!$C$10*C10</f>
@@ -17837,15 +17840,15 @@
         <v>58</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
     </row>
     <row r="16" s="1" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="C16" s="19" t="n">
         <f aca="false">DATOS!$C$22*C6</f>
@@ -17855,15 +17858,15 @@
         <v>58</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
     </row>
     <row r="17" s="1" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="C17" s="19" t="n">
         <f aca="false">DATOS!$C$23*C6</f>
@@ -17873,15 +17876,15 @@
         <v>58</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="C18" s="19" t="n">
         <f aca="false">DATOS!$C$52</f>
@@ -17891,10 +17894,10 @@
         <v>58</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
@@ -18011,12 +18014,12 @@
     </row>
     <row r="20" s="1" customFormat="true" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="31" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="true" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="32" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18024,16 +18027,16 @@
         <v>116</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
@@ -18093,7 +18096,7 @@
     </row>
     <row r="23" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="C23" s="7" t="n">
         <v>60.0901</v>
@@ -18105,7 +18108,7 @@
         <v>1970.905</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18122,7 +18125,7 @@
         <v>901.867</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18139,7 +18142,7 @@
         <v>729.797</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18156,7 +18159,7 @@
         <v>1621.809</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18173,7 +18176,7 @@
         <v>91.241</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18190,7 +18193,7 @@
         <v>676.532</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18207,12 +18210,12 @@
         <v>73.128</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="6" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="C30" s="7" t="n">
         <v>6</v>
@@ -18224,12 +18227,12 @@
         <v>25.471</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
     </row>
     <row r="31" s="1" customFormat="true" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="6" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="C31" s="7" t="n">
         <v>13.2</v>
@@ -18241,7 +18244,7 @@
         <v>180.118</v>
       </c>
       <c r="F31" s="10" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="G31" s="0"/>
       <c r="H31" s="0"/>
@@ -18301,7 +18304,7 @@
     </row>
     <row r="32" s="1" customFormat="true" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="6" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C32" s="7" t="n">
         <v>64.0861</v>
@@ -18313,12 +18316,12 @@
         <v>101.05</v>
       </c>
       <c r="F32" s="10" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
     </row>
     <row r="33" s="1" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="6" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="C33" s="7" t="n">
         <v>104.1</v>
@@ -18330,12 +18333,12 @@
         <v>123.108</v>
       </c>
       <c r="F33" s="10" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
     </row>
     <row r="34" s="1" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="6" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="C34" s="7" t="n">
         <v>146.2814</v>
@@ -18347,12 +18350,12 @@
         <v>145.157</v>
       </c>
       <c r="F34" s="10" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="6" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="C35" s="7" t="n">
         <v>21.5662</v>
@@ -18364,12 +18367,12 @@
         <v>33.438</v>
       </c>
       <c r="F35" s="10" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
     </row>
     <row r="36" s="1" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="6" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="C36" s="11" t="n">
         <f aca="false">SUM(C23:C35)</f>
@@ -18381,7 +18384,7 @@
         <v>6673.621</v>
       </c>
       <c r="F36" s="10" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
     </row>
     <row r="37" s="1" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18393,7 +18396,7 @@
     </row>
     <row r="38" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="31" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
@@ -18470,17 +18473,17 @@
     </row>
     <row r="40" s="1" customFormat="true" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="6" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="C40" s="11" t="n">
         <f aca="false">E36/1000</f>
         <v>6.673621</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="F40" s="10" t="s">
         <v>41</v>
@@ -18550,13 +18553,13 @@
         <v>3.1159296</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="F41" s="10" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
     </row>
     <row r="42" s="1" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18568,49 +18571,49 @@
         <v>2.213047512</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="F42" s="10" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
     </row>
     <row r="43" s="1" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="6" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="C43" s="11" t="n">
         <f aca="false">C18/1000</f>
         <v>0.3978</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="F43" s="10" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="6" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="C44" s="11" t="n">
         <f aca="false">C17/1000</f>
         <v>0</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="F44" s="10" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
@@ -18670,20 +18673,20 @@
     </row>
     <row r="45" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="6" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="C45" s="11" t="n">
         <f aca="false">SUM(C40:C44)</f>
         <v>12.400398112</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="F45" s="10" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
@@ -18743,19 +18746,19 @@
     </row>
     <row r="46" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="6" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="C46" s="11" t="n">
-        <v>12.41839</v>
+        <v>12.33062</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="F46" s="10" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18767,7 +18770,7 @@
     </row>
     <row r="48" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="31" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18789,7 +18792,7 @@
     </row>
     <row r="50" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="6" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="C50" s="11" t="n">
         <v>0.4</v>
@@ -18798,15 +18801,15 @@
         <v>41</v>
       </c>
       <c r="E50" s="9" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="F50" s="10" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="6" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="C51" s="11" t="n">
         <v>1</v>
@@ -18815,15 +18818,15 @@
         <v>41</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="F51" s="10" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="6" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="C52" s="11" t="n">
         <v>3</v>
@@ -18832,32 +18835,32 @@
         <v>41</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="F52" s="10" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B53" s="6" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="C53" s="11" t="n">
         <v>0.6</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="F53" s="10" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B54" s="6" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="C54" s="11" t="n">
         <v>7</v>
@@ -18866,15 +18869,15 @@
         <v>41</v>
       </c>
       <c r="E54" s="9" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="F54" s="10" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B55" s="6" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="C55" s="11" t="n">
         <v>0.085</v>
@@ -18883,15 +18886,15 @@
         <v>41</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="F55" s="10" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B56" s="6" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="C56" s="11" t="n">
         <f aca="false">DATOS!$C$15</f>
@@ -18901,7 +18904,7 @@
         <v>27</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="F56" s="10" t="s">
         <v>83</v>
@@ -18909,25 +18912,25 @@
     </row>
     <row r="57" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B57" s="6" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="C57" s="11" t="n">
         <f aca="false">C55*C56^0.75</f>
         <v>0.493323900968996</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="F57" s="10" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="6" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="C58" s="11" t="n">
         <f aca="false">C50*C51*C52/C54*(C53/MAX(C57,C53))^(2/3)</f>
@@ -18937,7 +18940,7 @@
         <v>41</v>
       </c>
       <c r="E58" s="9" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="F58" s="10" t="s">
         <v>83</v>
@@ -18945,153 +18948,153 @@
     </row>
     <row r="59" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B59" s="6" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="C59" s="11" t="n">
-        <v>0.61943</v>
+        <v>0.61658</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="F59" s="10" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B60" s="6" t="s">
+        <v>735</v>
+      </c>
+      <c r="C60" s="11" t="n">
+        <v>0.38161</v>
+      </c>
+      <c r="D60" s="8" t="s">
+        <v>721</v>
+      </c>
+      <c r="E60" s="9" t="s">
+        <v>736</v>
+      </c>
+      <c r="F60" s="10" t="s">
         <v>734</v>
-      </c>
-      <c r="C60" s="11" t="n">
-        <v>0.38249</v>
-      </c>
-      <c r="D60" s="8" t="s">
-        <v>720</v>
-      </c>
-      <c r="E60" s="9" t="s">
-        <v>735</v>
-      </c>
-      <c r="F60" s="10" t="s">
-        <v>733</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B61" s="6" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="C61" s="11" t="n">
-        <v>2082.83504</v>
+        <v>2068.11409</v>
       </c>
       <c r="D61" s="8" t="s">
         <v>58</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="F61" s="10" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="6" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="C62" s="11" t="n">
-        <v>2128.86686</v>
+        <v>2113.82057</v>
       </c>
       <c r="D62" s="8" t="s">
         <v>58</v>
       </c>
       <c r="E62" s="9" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="F62" s="10" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="6" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="C63" s="11" t="n">
-        <v>1874.55153</v>
+        <v>1861.30268</v>
       </c>
       <c r="D63" s="8" t="s">
         <v>58</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="F63" s="10" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="6" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="C64" s="11" t="n">
-        <v>1915.98017</v>
+        <v>1902.43851</v>
       </c>
       <c r="D64" s="8" t="s">
         <v>58</v>
       </c>
       <c r="E64" s="9" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="F64" s="10" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="6" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="C65" s="11" t="n">
-        <v>1708.31557</v>
+        <v>1694.76348</v>
       </c>
       <c r="D65" s="8" t="s">
         <v>58</v>
       </c>
       <c r="E65" s="9" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="F65" s="10" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="6" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="C66" s="11" t="n">
-        <v>1881.58154</v>
+        <v>1863.55753</v>
       </c>
       <c r="D66" s="8" t="s">
         <v>58</v>
       </c>
       <c r="E66" s="9" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="F66" s="10" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="6" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="C67" s="11" t="n">
         <f aca="false">MAX(1,C63/C65)</f>
-        <v>1.09730986646688</v>
+        <v>1.0982669274889</v>
       </c>
       <c r="D67" s="8" t="s">
         <v>41</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>83</v>
@@ -19099,17 +19102,17 @@
     </row>
     <row r="68" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="6" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="C68" s="11" t="n">
         <f aca="false">MAX(1,C64/C66)</f>
-        <v>1.01828176418015</v>
+        <v>1.02086384743915</v>
       </c>
       <c r="D68" s="8" t="s">
         <v>41</v>
       </c>
       <c r="E68" s="9" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="F68" s="10" t="s">
         <v>83</v>

</xml_diff>

<commit_message>
002 3.0: modos y peso dinámico del .ANL 3.0 en la hoja de sismo
Corrida del usuario sin errores: 6673.62 kg de take off, ningún FAIL,
ratio máximo 0.933 (largueros de muro claro 2-3), deriva 0.01406 (0.937
del límite 0.015), DYNAMIC WEIGHT 12330.62 kg, T1 = 0.61669 s. Con los 43
modos del .ANL la hoja de sismo da factores X 1.0979 / Z 1.0218, que pasan
al STD. Se actualizan áreas tributarias (sección 5 y notas), desglose y
reacciones.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DbpSpoM7qi5cJ9LMKpwgVv
</commit_message>
<xml_diff>
--- a/002/002_AreasTributarias_NOSE_DOCK_H5_H6_3.0.xlsx
+++ b/002/002_AreasTributarias_NOSE_DOCK_H5_H6_3.0.xlsx
@@ -1933,7 +1933,7 @@
     <t xml:space="preserve">SELFWEIGHT Z 1</t>
   </si>
   <si>
-    <t xml:space="preserve">CASO 4: estas líneas van ANTES del SPECTRUM. CASOS 5 A 7 usan la masa del caso 4. Cubierta y muros quedan como JOINT LOAD en las cabezas de columna. CUT OFF MODE SHAPE = 43; participación modal acumulada X = 91.66% y Z = 96.10%. Muros A y B de 0.30 m al alero con la mitad de cada claro (Z 0 a 4, 4 a 12 y 12 a 16 m); muro 1 partido a la mitad en X = 5.04 m, cada mitad con sus vanos, una al nodo 7 y otra al nodo 8; media cortina en cada jamba. Muros y cortina: 5.85 kg/m² × 378.30 m² + 397.8 kg = 2,610.84 kg.</t>
+    <t xml:space="preserve">CASO 4: estas líneas van ANTES del SPECTRUM. CASOS 5 A 7 usan la masa del caso 4. Cubierta y muros quedan como JOINT LOAD en las cabezas de columna. CUT OFF MODE SHAPE = 43; participación modal acumulada X = 91.64% y Z = 95.91%. Muros A y B de 0.30 m al alero con la mitad de cada claro (Z 0 a 4, 4 a 12 y 12 a 16 m); muro 1 partido a la mitad en X = 5.04 m, cada mitad con sus vanos, una al nodo 7 y otra al nodo 8; media cortina en cada jamba. Muros y cortina: 5.85 kg/m² × 378.30 m² + 397.8 kg = 2,610.84 kg.</t>
   </si>
   <si>
     <t xml:space="preserve">RESUMEN — ÁREAS, CARGAS TOTALES Y PESO SÍSMICO W</t>
@@ -2164,10 +2164,10 @@
     <t xml:space="preserve">W dinámico de STAAD — dirección X</t>
   </si>
   <si>
-    <t xml:space="preserve">Peso dinámico del motor de análisis para la 3.0 (43 modos); igual en X y en Z. Se confirma con la corrida de STAAD.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">.STD 3.0 · motor de análisis</t>
+    <t xml:space="preserve">DYNAMIC WEIGHT de la corrida 3.0 (43 modos); igual en X y en Z.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">.ANL 3.0</t>
   </si>
   <si>
     <t xml:space="preserve">5. CORTANTE MÍNIMO NTDS §5.4.1(3) → FACTOR DEL SPECTRUM EN STAAD</t>
@@ -2227,16 +2227,16 @@
     <t xml:space="preserve">T_B en X (modo con más masa en X)</t>
   </si>
   <si>
-    <t xml:space="preserve">Modo 1: mayor participación en X (81.76%).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">motor 3.0 (43 modos)</t>
+    <t xml:space="preserve">Modo 1: mayor participación en X (81.79%).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">.ANL 3.0 (43 modos)</t>
   </si>
   <si>
     <t xml:space="preserve">T_B en Z (modo con más masa en Z)</t>
   </si>
   <si>
-    <t xml:space="preserve">Modo 7: mayor participación en Z (88.00%).</t>
+    <t xml:space="preserve">Modo 7: mayor participación en Z (87.91%).</t>
   </si>
   <si>
     <t xml:space="preserve">V_est en X = máx(Cs(T_B), 0.8·Cs(T_A))·W</t>
@@ -2260,25 +2260,25 @@
     <t xml:space="preserve">V modal en X (sin factor)</t>
   </si>
   <si>
-    <t xml:space="preserve">SRSS de los 43 modos del motor, sin factor (hoja de sismo K237).</t>
+    <t xml:space="preserve">SRSS de los 43 modos de la corrida 3.0, sin factor (hoja de sismo K237).</t>
   </si>
   <si>
     <t xml:space="preserve">V modal en Z (sin factor)</t>
   </si>
   <si>
-    <t xml:space="preserve">SRSS de los 43 modos del motor, sin factor (hoja de sismo L237).</t>
+    <t xml:space="preserve">SRSS de los 43 modos de la corrida 3.0, sin factor (hoja de sismo L237).</t>
   </si>
   <si>
     <t xml:space="preserve">Factor del SPECTRUM en X</t>
   </si>
   <si>
-    <t xml:space="preserve">Factor mínimo requerido en X; el .STD usa 1.0983.</t>
+    <t xml:space="preserve">Factor mínimo requerido en X; el .STD usa 1.0979.</t>
   </si>
   <si>
     <t xml:space="preserve">Factor del SPECTRUM en Z</t>
   </si>
   <si>
-    <t xml:space="preserve">Factor mínimo requerido en Z; el .STD usa 1.0209.</t>
+    <t xml:space="preserve">Factor mínimo requerido en Z; el .STD usa 1.0218.</t>
   </si>
 </sst>
 </file>
@@ -18951,7 +18951,7 @@
         <v>732</v>
       </c>
       <c r="C59" s="11" t="n">
-        <v>0.61658</v>
+        <v>0.61669</v>
       </c>
       <c r="D59" s="8" t="s">
         <v>721</v>
@@ -18968,7 +18968,7 @@
         <v>735</v>
       </c>
       <c r="C60" s="11" t="n">
-        <v>0.38161</v>
+        <v>0.38231</v>
       </c>
       <c r="D60" s="8" t="s">
         <v>721</v>
@@ -19053,7 +19053,7 @@
         <v>743</v>
       </c>
       <c r="C65" s="11" t="n">
-        <v>1694.76348</v>
+        <v>1695.34887</v>
       </c>
       <c r="D65" s="8" t="s">
         <v>58</v>
@@ -19070,7 +19070,7 @@
         <v>745</v>
       </c>
       <c r="C66" s="11" t="n">
-        <v>1863.55753</v>
+        <v>1861.81363</v>
       </c>
       <c r="D66" s="8" t="s">
         <v>58</v>
@@ -19088,7 +19088,7 @@
       </c>
       <c r="C67" s="11" t="n">
         <f aca="false">MAX(1,C63/C65)</f>
-        <v>1.0982669274889</v>
+        <v>1.09788770496541</v>
       </c>
       <c r="D67" s="8" t="s">
         <v>41</v>
@@ -19106,7 +19106,7 @@
       </c>
       <c r="C68" s="11" t="n">
         <f aca="false">MAX(1,C64/C66)</f>
-        <v>1.02086384743915</v>
+        <v>1.02182005725245</v>
       </c>
       <c r="D68" s="8" t="s">
         <v>41</v>

</xml_diff>